<commit_message>
Fix CMA brand key in Book H1 tags
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Book_H1_tags.xlsx
+++ b/Book_H1_tags.xlsx
@@ -5150,48 +5150,56 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="4" t="inlineStr">
+      <c r="A177" t="inlineStr">
         <is>
           <t>Cma Dish Machines</t>
         </is>
       </c>
-      <c r="B177" s="4" t="inlineStr">
+      <c r="B177" t="inlineStr">
         <is>
           <t>13417.92</t>
         </is>
       </c>
-      <c r="C177" s="4" t="inlineStr"/>
-      <c r="D177" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E177" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>Cma Dish Machines Dishwasher Heater Control Thermostat (12kW) - 13417.92</t>
+        </is>
+      </c>
+      <c r="D177" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>GWX-200, EST models</t>
         </is>
       </c>
     </row>
     <row r="178">
-      <c r="A178" s="4" t="inlineStr">
+      <c r="A178" t="inlineStr">
         <is>
           <t>Cma Dish Machines</t>
         </is>
       </c>
-      <c r="B178" s="4" t="inlineStr">
+      <c r="B178" t="inlineStr">
         <is>
           <t>13417.94</t>
         </is>
       </c>
-      <c r="C178" s="4" t="inlineStr"/>
-      <c r="D178" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E178" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Cma Dish Machines Dishwasher Thermostat Assembly - 13417.94</t>
+        </is>
+      </c>
+      <c r="D178" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>Parts Town: fits five CMA models</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Complete Book H1 tags (all 418 parts)
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Book_H1_tags.xlsx
+++ b/Book_H1_tags.xlsx
@@ -29,7 +29,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -46,11 +46,6 @@
         <fgColor rgb="00F8CBAD"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -64,12 +59,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -10899,646 +10893,750 @@
       </c>
     </row>
     <row r="392">
-      <c r="A392" s="4" t="inlineStr">
+      <c r="A392" t="inlineStr">
         <is>
           <t>Scotsman</t>
         </is>
       </c>
-      <c r="B392" s="4" t="inlineStr">
+      <c r="B392" t="inlineStr">
         <is>
           <t>R620314803</t>
         </is>
       </c>
-      <c r="C392" s="4" t="inlineStr"/>
-      <c r="D392" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E392" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Scotsman Ice Machine Agitation Timer 120V - R620314803</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E392" t="inlineStr">
+        <is>
+          <t>Amazon, Parts Town and FixIce (ID150/ID200 dispensers)</t>
         </is>
       </c>
     </row>
     <row r="393">
-      <c r="A393" s="4" t="inlineStr">
+      <c r="A393" t="inlineStr">
         <is>
           <t>Sharp</t>
         </is>
       </c>
-      <c r="B393" s="4" t="inlineStr">
+      <c r="B393" t="inlineStr">
         <is>
           <t>FGLSPA069WRFZ</t>
         </is>
       </c>
-      <c r="C393" s="4" t="inlineStr"/>
-      <c r="D393" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E393" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>Sharp Microwave Oven Oven Tray Assembly - FGLSPA069WRFZ</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E393" t="inlineStr">
+        <is>
+          <t>Sharp commercial microwaves RCD1800M/RCD2200M; several sellers</t>
         </is>
       </c>
     </row>
     <row r="394">
-      <c r="A394" s="4" t="inlineStr">
+      <c r="A394" s="2" t="inlineStr">
         <is>
           <t>Sony</t>
         </is>
       </c>
-      <c r="B394" s="4" t="inlineStr">
+      <c r="B394" s="2" t="inlineStr">
         <is>
           <t>A-5014-378-A</t>
         </is>
       </c>
-      <c r="C394" s="4" t="inlineStr"/>
-      <c r="D394" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E394" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C394" s="2" t="inlineStr">
+        <is>
+          <t>Sony TV ONT J Board - A-5014-378-A</t>
+        </is>
+      </c>
+      <c r="D394" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E394" s="2" t="inlineStr">
+        <is>
+          <t>Sellers disagree on name (ONT J board vs Compl Svc ONTJ_NE); XBR-75/85Z8H</t>
         </is>
       </c>
     </row>
     <row r="395">
-      <c r="A395" s="4" t="inlineStr">
+      <c r="A395" s="3" t="inlineStr">
         <is>
           <t>Sony</t>
         </is>
       </c>
-      <c r="B395" s="4" t="inlineStr">
+      <c r="B395" s="3" t="inlineStr">
         <is>
           <t>A-5057-109-A</t>
         </is>
       </c>
-      <c r="C395" s="4" t="inlineStr"/>
-      <c r="D395" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E395" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C395" s="3" t="inlineStr"/>
+      <c r="D395" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E395" s="3" t="inlineStr">
+        <is>
+          <t>Searched "A-5057-109-A" Sony; no listing found, only neighbouring A-5057 numbers</t>
         </is>
       </c>
     </row>
     <row r="396">
-      <c r="A396" s="4" t="inlineStr">
+      <c r="A396" s="2" t="inlineStr">
         <is>
           <t>Speed Queen</t>
         </is>
       </c>
-      <c r="B396" s="4" t="inlineStr">
+      <c r="B396" s="2" t="inlineStr">
         <is>
           <t>70482901</t>
         </is>
       </c>
-      <c r="C396" s="4" t="inlineStr"/>
-      <c r="D396" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E396" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C396" s="2" t="inlineStr">
+        <is>
+          <t>Speed Queen Washer Door Catch Kit - 70482901</t>
+        </is>
+      </c>
+      <c r="D396" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E396" s="2" t="inlineStr">
+        <is>
+          <t>Alliance Laundry store lists it for washers and dryers</t>
         </is>
       </c>
     </row>
     <row r="397">
-      <c r="A397" s="4" t="inlineStr">
+      <c r="A397" t="inlineStr">
         <is>
           <t>Turbochef</t>
         </is>
       </c>
-      <c r="B397" s="4" t="inlineStr">
+      <c r="B397" t="inlineStr">
         <is>
           <t>103566</t>
         </is>
       </c>
-      <c r="C397" s="4" t="inlineStr"/>
-      <c r="D397" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E397" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Turbochef Oven Fuse Block 3-Pole 600V 30A - 103566</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E397" t="inlineStr">
+        <is>
+          <t>Parts Town and Encore service manual</t>
         </is>
       </c>
     </row>
     <row r="398">
-      <c r="A398" s="4" t="inlineStr">
+      <c r="A398" s="2" t="inlineStr">
         <is>
           <t>Turbochef</t>
         </is>
       </c>
-      <c r="B398" s="4" t="inlineStr">
+      <c r="B398" s="2" t="inlineStr">
         <is>
           <t>301365</t>
         </is>
       </c>
-      <c r="C398" s="4" t="inlineStr"/>
-      <c r="D398" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E398" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C398" s="2" t="inlineStr">
+        <is>
+          <t>Turbochef Oven Temperature Sensor Assembly - 301365</t>
+        </is>
+      </c>
+      <c r="D398" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E398" s="2" t="inlineStr">
+        <is>
+          <t>Single Parts Town listing; discontinued</t>
         </is>
       </c>
     </row>
     <row r="399">
-      <c r="A399" s="4" t="inlineStr">
+      <c r="A399" s="3" t="inlineStr">
         <is>
           <t>Turbochef</t>
         </is>
       </c>
-      <c r="B399" s="4" t="inlineStr">
+      <c r="B399" s="3" t="inlineStr">
         <is>
           <t>301684</t>
         </is>
       </c>
-      <c r="C399" s="4" t="inlineStr"/>
-      <c r="D399" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E399" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C399" s="3" t="inlineStr">
+        <is>
+          <t>Turbochef Oven Power Output Stage Assembly, 3 Phase - 301684</t>
+        </is>
+      </c>
+      <c r="D399" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E399" s="3" t="inlineStr">
+        <is>
+          <t>Single old catalog page; price/details unconfirmed</t>
         </is>
       </c>
     </row>
     <row r="400">
-      <c r="A400" s="4" t="inlineStr">
+      <c r="A400" t="inlineStr">
         <is>
           <t>Turbochef</t>
         </is>
       </c>
-      <c r="B400" s="4" t="inlineStr">
+      <c r="B400" t="inlineStr">
         <is>
           <t>CON-3046</t>
         </is>
       </c>
-      <c r="C400" s="4" t="inlineStr"/>
-      <c r="D400" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E400" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Turbochef Oven Control Board Service Kit - CON-3046</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E400" t="inlineStr">
+        <is>
+          <t>Many sellers; HHD / Sage T models</t>
         </is>
       </c>
     </row>
     <row r="401">
-      <c r="A401" s="4" t="inlineStr">
+      <c r="A401" s="2" t="inlineStr">
         <is>
           <t>Turbochef</t>
         </is>
       </c>
-      <c r="B401" s="4" t="inlineStr">
+      <c r="B401" s="2" t="inlineStr">
         <is>
           <t>ECO-3212</t>
         </is>
       </c>
-      <c r="C401" s="4" t="inlineStr"/>
-      <c r="D401" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E401" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C401" s="2" t="inlineStr">
+        <is>
+          <t>Turbochef Oven Service Kit, Phoenix to HLUI (ECO) - ECO-3212</t>
+        </is>
+      </c>
+      <c r="D401" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E401" s="2" t="inlineStr">
+        <is>
+          <t>Single Turbochef Canada listing; I1-3212 stirrer is a different part</t>
         </is>
       </c>
     </row>
     <row r="402">
-      <c r="A402" s="4" t="inlineStr">
+      <c r="A402" t="inlineStr">
         <is>
           <t>Turbochef</t>
         </is>
       </c>
-      <c r="B402" s="4" t="inlineStr">
+      <c r="B402" t="inlineStr">
         <is>
           <t>ENC-3005-1</t>
         </is>
       </c>
-      <c r="C402" s="4" t="inlineStr"/>
-      <c r="D402" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E402" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>Turbochef Oven Encore Light Ring Service Kit - ENC-3005-1</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E402" t="inlineStr">
+        <is>
+          <t>Fits Encore / Encore 2; many sellers</t>
         </is>
       </c>
     </row>
     <row r="403">
-      <c r="A403" s="4" t="inlineStr">
+      <c r="A403" s="2" t="inlineStr">
         <is>
           <t>Turbochef</t>
         </is>
       </c>
-      <c r="B403" s="4" t="inlineStr">
+      <c r="B403" s="2" t="inlineStr">
         <is>
           <t>ENC-3010-1</t>
         </is>
       </c>
-      <c r="C403" s="4" t="inlineStr"/>
-      <c r="D403" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E403" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C403" s="2" t="inlineStr">
+        <is>
+          <t>Turbochef Oven Capacitor 2500V 50/60Hz - ENC-3010-1</t>
+        </is>
+      </c>
+      <c r="D403" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E403" s="2" t="inlineStr">
+        <is>
+          <t>Parts Town, Webstaurant and eBay; no model list</t>
         </is>
       </c>
     </row>
     <row r="404">
-      <c r="A404" s="4" t="inlineStr">
+      <c r="A404" t="inlineStr">
         <is>
           <t>Turbochef</t>
         </is>
       </c>
-      <c r="B404" s="4" t="inlineStr">
+      <c r="B404" t="inlineStr">
         <is>
           <t>ENC-3011</t>
         </is>
       </c>
-      <c r="C404" s="4" t="inlineStr"/>
-      <c r="D404" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E404" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Turbochef Oven 4.3" TFT Display Board Service Kit - ENC-3011</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E404" t="inlineStr">
+        <is>
+          <t>Encore / Encore 2 / NGO; many sellers</t>
         </is>
       </c>
     </row>
     <row r="405">
-      <c r="A405" s="4" t="inlineStr">
+      <c r="A405" t="inlineStr">
         <is>
           <t>Turbochef</t>
         </is>
       </c>
-      <c r="B405" s="4" t="inlineStr">
+      <c r="B405" t="inlineStr">
         <is>
           <t>ENC-3022</t>
         </is>
       </c>
-      <c r="C405" s="4" t="inlineStr"/>
-      <c r="D405" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E405" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Turbochef Oven Door Hinge Kit with Springs (Set of 2) - ENC-3022</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E405" t="inlineStr">
+        <is>
+          <t>Many sellers agree</t>
         </is>
       </c>
     </row>
     <row r="406">
-      <c r="A406" s="4" t="inlineStr">
+      <c r="A406" s="3" t="inlineStr">
         <is>
           <t>Turbochef</t>
         </is>
       </c>
-      <c r="B406" s="4" t="inlineStr">
+      <c r="B406" s="3" t="inlineStr">
         <is>
           <t>HCT-4401</t>
         </is>
       </c>
-      <c r="C406" s="4" t="inlineStr"/>
-      <c r="D406" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E406" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C406" s="3" t="inlineStr">
+        <is>
+          <t>Turbochef Oven Low Voltage Harness - HCT-4401</t>
+        </is>
+      </c>
+      <c r="D406" s="3" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E406" s="3" t="inlineStr">
+        <is>
+          <t>Two listings only, no price or fit information</t>
         </is>
       </c>
     </row>
     <row r="407">
-      <c r="A407" s="4" t="inlineStr">
+      <c r="A407" t="inlineStr">
         <is>
           <t>Turbochef</t>
         </is>
       </c>
-      <c r="B407" s="4" t="inlineStr">
+      <c r="B407" t="inlineStr">
         <is>
           <t>HHB-3204</t>
         </is>
       </c>
-      <c r="C407" s="4" t="inlineStr"/>
-      <c r="D407" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E407" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Turbochef Oven Display Service Kit (HHB) - HHB-3204</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E407" t="inlineStr">
+        <is>
+          <t>Many sellers agree</t>
         </is>
       </c>
     </row>
     <row r="408">
-      <c r="A408" s="4" t="inlineStr">
+      <c r="A408" t="inlineStr">
         <is>
           <t>Turbochef</t>
         </is>
       </c>
-      <c r="B408" s="4" t="inlineStr">
+      <c r="B408" t="inlineStr">
         <is>
           <t>HHC-4120</t>
         </is>
       </c>
-      <c r="C408" s="4" t="inlineStr"/>
-      <c r="D408" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E408" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>Turbochef Conveyor Oven Conveyor Gear Motor 1/50 HP 208/230V - HHC-4120</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E408" t="inlineStr">
+        <is>
+          <t>HHC series; several sellers</t>
         </is>
       </c>
     </row>
     <row r="409">
-      <c r="A409" s="4" t="inlineStr">
+      <c r="A409" t="inlineStr">
         <is>
           <t>Turbochef</t>
         </is>
       </c>
-      <c r="B409" s="4" t="inlineStr">
+      <c r="B409" t="inlineStr">
         <is>
           <t>HHD-3003</t>
         </is>
       </c>
-      <c r="C409" s="4" t="inlineStr"/>
-      <c r="D409" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E409" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>Turbochef Oven Heater Assembly Service Kit (HHD) - HHD-3003</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E409" t="inlineStr">
+        <is>
+          <t>HHD double batch ovens; many sellers</t>
         </is>
       </c>
     </row>
     <row r="410">
-      <c r="A410" s="4" t="inlineStr">
+      <c r="A410" s="2" t="inlineStr">
         <is>
           <t>Turbochef</t>
         </is>
       </c>
-      <c r="B410" s="4" t="inlineStr">
+      <c r="B410" s="2" t="inlineStr">
         <is>
           <t>I1-3201-10</t>
         </is>
       </c>
-      <c r="C410" s="4" t="inlineStr"/>
-      <c r="D410" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E410" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C410" s="2" t="inlineStr">
+        <is>
+          <t>Turbochef Oven Oven Door, Black - I1-3201-10</t>
+        </is>
+      </c>
+      <c r="D410" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E410" s="2" t="inlineStr">
+        <is>
+          <t>AllPoints and Turbochef Canada; two sellers</t>
         </is>
       </c>
     </row>
     <row r="411">
-      <c r="A411" s="4" t="inlineStr">
+      <c r="A411" t="inlineStr">
         <is>
           <t>Turbochef</t>
         </is>
       </c>
-      <c r="B411" s="4" t="inlineStr">
+      <c r="B411" t="inlineStr">
         <is>
           <t>I1-9166</t>
         </is>
       </c>
-      <c r="C411" s="4" t="inlineStr"/>
-      <c r="D411" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E411" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Turbochef Oven Cooking Basket, Solid PTFE 11.5" x 8.5" - I1-9166</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E411" t="inlineStr">
+        <is>
+          <t>Several sellers; obsolete, replaced by 105696</t>
         </is>
       </c>
     </row>
     <row r="412">
-      <c r="A412" s="4" t="inlineStr">
+      <c r="A412" t="inlineStr">
         <is>
           <t>Turbochef</t>
         </is>
       </c>
-      <c r="B412" s="4" t="inlineStr">
+      <c r="B412" t="inlineStr">
         <is>
           <t>I3-3231</t>
         </is>
       </c>
-      <c r="C412" s="4" t="inlineStr"/>
-      <c r="D412" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E412" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Turbochef Oven Touchscreen Service Kit, Phoenix to HLUI (i3) - I3-3231</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E412" t="inlineStr">
+        <is>
+          <t>Many sellers agree</t>
         </is>
       </c>
     </row>
     <row r="413">
-      <c r="A413" s="4" t="inlineStr">
+      <c r="A413" s="2" t="inlineStr">
         <is>
           <t>Turbochef</t>
         </is>
       </c>
-      <c r="B413" s="4" t="inlineStr">
+      <c r="B413" s="2" t="inlineStr">
         <is>
           <t>I5-9378</t>
         </is>
       </c>
-      <c r="C413" s="4" t="inlineStr"/>
-      <c r="D413" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E413" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C413" s="2" t="inlineStr">
+        <is>
+          <t>Turbochef Oven Capacitor Jumper Wire - I5-9378</t>
+        </is>
+      </c>
+      <c r="D413" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E413" s="2" t="inlineStr">
+        <is>
+          <t>Parts Town and Middleby Advantage; one result is a different part (I3-9378 heater)</t>
         </is>
       </c>
     </row>
     <row r="414">
-      <c r="A414" s="4" t="inlineStr">
+      <c r="A414" t="inlineStr">
         <is>
           <t>Turbochef</t>
         </is>
       </c>
-      <c r="B414" s="4" t="inlineStr">
+      <c r="B414" t="inlineStr">
         <is>
           <t>NGC-3005</t>
         </is>
       </c>
-      <c r="C414" s="4" t="inlineStr"/>
-      <c r="D414" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E414" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>Turbochef Oven Dual 40A Solid State Relay 120/240V - NGC-3005</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>Many sellers; NGC/HHB/i3 ovens</t>
         </is>
       </c>
     </row>
     <row r="415">
-      <c r="A415" s="4" t="inlineStr">
+      <c r="A415" s="2" t="inlineStr">
         <is>
           <t>Turbochef</t>
         </is>
       </c>
-      <c r="B415" s="4" t="inlineStr">
+      <c r="B415" s="2" t="inlineStr">
         <is>
           <t>PLE-3228</t>
         </is>
       </c>
-      <c r="C415" s="4" t="inlineStr"/>
-      <c r="D415" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E415" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C415" s="2" t="inlineStr">
+        <is>
+          <t>Turbochef Oven Switch Service Kit (Plexor) - PLE-3228</t>
+        </is>
+      </c>
+      <c r="D415" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E415" s="2" t="inlineStr">
+        <is>
+          <t>Parts Town Plexor A3 pages; description is generic</t>
         </is>
       </c>
     </row>
     <row r="416">
-      <c r="A416" s="4" t="inlineStr">
+      <c r="A416" t="inlineStr">
         <is>
           <t>U-Line</t>
         </is>
       </c>
-      <c r="B416" s="4" t="inlineStr">
+      <c r="B416" t="inlineStr">
         <is>
           <t>80-54138-00</t>
         </is>
       </c>
-      <c r="C416" s="4" t="inlineStr"/>
-      <c r="D416" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E416" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>U-Line Refrigerator Condenser Fan Motor - 80-54138-00</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E416" t="inlineStr">
+        <is>
+          <t>Several sellers and model parts lists</t>
         </is>
       </c>
     </row>
     <row r="417">
-      <c r="A417" s="4" t="inlineStr">
+      <c r="A417" s="2" t="inlineStr">
         <is>
           <t>U-Line</t>
         </is>
       </c>
-      <c r="B417" s="4" t="inlineStr">
+      <c r="B417" s="2" t="inlineStr">
         <is>
           <t>80-54149-00</t>
         </is>
       </c>
-      <c r="C417" s="4" t="inlineStr"/>
-      <c r="D417" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E417" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C417" s="2" t="inlineStr">
+        <is>
+          <t>U-Line Refrigerator Compressor Electrical Kit (Compressor Electricals Only) - 80-54149-00</t>
+        </is>
+      </c>
+      <c r="D417" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E417" s="2" t="inlineStr">
+        <is>
+          <t>U-Line parts documents; limited seller listings</t>
         </is>
       </c>
     </row>
     <row r="418">
-      <c r="A418" s="4" t="inlineStr">
+      <c r="A418" s="3" t="inlineStr">
         <is>
           <t>Whirlpool</t>
         </is>
       </c>
-      <c r="B418" s="4" t="inlineStr">
+      <c r="B418" s="3" t="inlineStr">
         <is>
           <t>300248</t>
         </is>
       </c>
-      <c r="C418" s="4" t="inlineStr"/>
-      <c r="D418" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E418" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C418" s="3" t="inlineStr"/>
+      <c r="D418" s="3" t="inlineStr">
+        <is>
+          <t>Needs review</t>
+        </is>
+      </c>
+      <c r="E418" s="3" t="inlineStr">
+        <is>
+          <t>Searched "300248" Whirlpool; no matching listing found</t>
         </is>
       </c>
     </row>
     <row r="419">
-      <c r="A419" s="4" t="inlineStr">
+      <c r="A419" t="inlineStr">
         <is>
           <t>York</t>
         </is>
       </c>
-      <c r="B419" s="4" t="inlineStr">
+      <c r="B419" t="inlineStr">
         <is>
           <t>S1-32649692000</t>
         </is>
       </c>
-      <c r="C419" s="4" t="inlineStr"/>
-      <c r="D419" s="4" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E419" s="4" t="inlineStr">
-        <is>
-          <t>Not searched: per-turn web search limit reached.</t>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>York Furnace Draft Inducer Combustion Blower Motor Assembly (90%) - S1-32649692000</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E419" t="inlineStr">
+        <is>
+          <t>Many sellers agree; fit lists vary</t>
         </is>
       </c>
     </row>

</xml_diff>